<commit_message>
Update EX HITACHI summary: drop IGCT, add packaging and gross weight
Confirmed with the sender's e-mail that no IGCT thyristors are part of
this shipment, so the IGCT category is removed.

- Quantities cross-checked against the e-mail and match: thyristors
  8541 30 00 = 18 + 12 = 30 pcs; diodes 8541 10 00 = 100 + 100 + 100 = 300 pcs
- Added packaging block for the export document / ATR: 1 pallet
  60 x 40 x 75 cm, total gross weight 77 kg, total net weight 60.20 kg
- Reworded the missing gross weight note on delivery note 0924453368:
  the 77 kg shipment gross is the figure to use for the export document

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BnK8TWbJrhHRLE4rErTTKo
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Energy_EX_HITACHI.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Energy_EX_HITACHI.xlsx
@@ -78,9 +78,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
-  <si>
-    <t xml:space="preserve">Souhrn zásilky EX HITACHI – tyristory / diody / IGCT tyristory</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
+  <si>
+    <t xml:space="preserve">Souhrn zásilky EX HITACHI – tyristory a diody</t>
   </si>
   <si>
     <t xml:space="preserve">Odesílatel: Hitachi Energy Czech Republic s.r.o., Na strži 1702/65, 140 00 Praha 4  |  Příjemce: Protek Teknik Elektrik Ticaret Ve Sanayi Ltd Sti, Türkiye</t>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">85413000</t>
   </si>
   <si>
-    <t xml:space="preserve">chybí</t>
+    <t xml:space="preserve">neuvedeno</t>
   </si>
   <si>
     <t xml:space="preserve">810679464</t>
@@ -194,40 +194,58 @@
     <t xml:space="preserve">Celkem tyristory</t>
   </si>
   <si>
-    <t xml:space="preserve">IGCT TYRISTORY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ŽÁDNÉ POLOŽKY – v předložených 4 fakturách nejsou žádné IGCT tyristory (řada 5SHY)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Celkem IGCT tyristory</t>
-  </si>
-  <si>
     <t xml:space="preserve">CELKEM ZÁSILKA</t>
   </si>
   <si>
+    <t xml:space="preserve">Balení a hmotnost zásilky (pro vývozní doklad / ATR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Počet kolli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 paleta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozměry palety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 × 40 × 75 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celková hrubá hmotnost zásilky (vč. palety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celková čistá hmotnost zboží (dle faktur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60,20 kg</t>
+  </si>
+  <si>
     <t xml:space="preserve">Poznámky</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Zásilka obsahuje pouze 2 HS kódy: 8541 10 00 (diody) a 8541 30 00 (tyristory, diaky, triaky a tyristory zapalované světlem).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2) IGCT TYRISTORY: v předložených 4 fakturách (810679463, 810679464, 810679483, 810679510) nejsou žádné IGCT tyristory. IGCT je u Hitachi Energy řada 5SHY – ta se v dokladech nevyskytuje. Pokud mají být IGCT součástí zásilky, chybí k nim faktura a packing list.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3) Hrubá hmotnost u položky 5STF 15F2040 (faktura 810679464 / dodací list 0924453368) je na dodacím listu uvedena jako 0 kg – údaj chybí a je nutné jej doplnit od odesílatele. Součty hrubé hmotnosti jsou proto o tuto položku nižší.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4) Faktura 810679463 obsahuje dvě položky téhož materiálu 5SDD 0135Z0401 (pol. 10 a 40), každá 100 ks / 14 kg net; v souhrnu jsou sloučeny do jednoho řádku (200 ks / 28 kg).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5) Čísla packing listů odpovídají číslům dodacích listů (Delivery Note) na dokladech Hitachi Energy; názvy souborů z e-mailu mají navíc koncovou číslici (např. 09244533391 = dodací list 0924453339).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6) Na žádost zadavatele NEBYLO v tomto souhrnu řešeno CBAM ani preferenční věta (COO).</t>
+    <t xml:space="preserve">1) Zásilka obsahuje pouze 2 HS kódy: 8541 10 00 (diody) a 8541 30 00 (tyristory, diaky, triaky a tyristory zapalované světlem). Oba kódy je nutné uvést na ATR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2) IGCT TYRISTORY nejsou součástí této zásilky – potvrzeno zadavatelem. Zásilka obsahuje pouze tyristory (5STF, 5STP) a diody (5SDD).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3) Kontrola množství proti e-mailu „Zásilka pro Protek Teknik + ATR“ souhlasí: tyristory 8541 30 00 = 18 + 12 ks = 30 ks; diody 8541 10 00 = 100 + 100 + 100 ks = 300 ks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4) Hrubá hmotnost u položky 5STF 15F2040 (faktura 810679464 / dodací list 0924453368) není na dodacím listu uvedena (je vytištěno 0 kg). Pro vývozní doklad se použije celková hrubá hmotnost zásilky 77 kg podle e-mailu; sloupcový součet hrubé hmotnosti z dodacích listů je proto pouze orientační.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5) Faktura 810679463 obsahuje dvě položky téhož materiálu 5SDD 0135Z0401 (pol. 10 a 40), každá 100 ks / 14 kg net; v souhrnu jsou sloučeny do jednoho řádku (200 ks / 28 kg). Spolu s fakturou 810679483 (100 ks) dává 300 ks diod dle e-mailu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6) Čísla packing listů odpovídají číslům dodacích listů (Delivery Note) na dokladech Hitachi Energy; názvy souborů z e-mailu mají navíc koncovou číslici (např. 09244533391 = dodací list 0924453339).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7) Na žádost zadavatele NEBYLO v tomto souhrnu řešeno CBAM ani preferenční věta (COO).</t>
   </si>
 </sst>
 </file>
@@ -494,22 +512,6 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -520,6 +522,22 @@
     </xf>
     <xf numFmtId="166" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -782,7 +800,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -1069,134 +1087,89 @@
       <c r="H15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20"/>
-      <c r="B17" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="20"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E19" s="17"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="25" t="n">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="21" t="n">
         <f aca="false">E9+E14</f>
         <v>330</v>
       </c>
-      <c r="F20" s="26" t="n">
+      <c r="F16" s="22" t="n">
         <f aca="false">F9+F14</f>
         <v>60.2</v>
       </c>
-      <c r="G20" s="26" t="n">
+      <c r="G16" s="22" t="n">
         <f aca="false">G9+G14</f>
         <v>58.92</v>
       </c>
-      <c r="H20" s="26" t="n">
+      <c r="H16" s="22" t="n">
         <f aca="false">H9+H14</f>
         <v>37146</v>
       </c>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27" t="s">
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="25"/>
+      <c r="C19" s="26" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="25"/>
+      <c r="C20" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-    </row>
-    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-    </row>
-    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+      <c r="B21" s="25"/>
+      <c r="C21" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="28"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="25"/>
+      <c r="C22" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
@@ -1210,7 +1183,7 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B26" s="28"/>
       <c r="C26" s="28"/>
@@ -1224,7 +1197,7 @@
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="28" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
@@ -1238,7 +1211,7 @@
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="28"/>
@@ -1250,15 +1223,58 @@
       <c r="I28" s="28"/>
       <c r="J28" s="28"/>
     </row>
+    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="28"/>
+    </row>
+    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+    </row>
+    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="28"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A23:J23"/>
+  <mergeCells count="8">
     <mergeCell ref="A24:J24"/>
     <mergeCell ref="A25:J25"/>
     <mergeCell ref="A26:J26"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A31:J31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>